<commit_message>
Updated Case 6, 7
</commit_message>
<xml_diff>
--- a/Data/Sample.xlsx
+++ b/Data/Sample.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rsk_a\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PyCode\nism\quiz_app\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E52E2A70-828C-4733-AFF1-BAE5C0964882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07703D48-C3EB-4210-81CA-C416C1CC412C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{B3B2EAEB-3D4F-44E9-A7BC-7C78BD8AFC15}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="5" xr2:uid="{B3B2EAEB-3D4F-44E9-A7BC-7C78BD8AFC15}"/>
   </bookViews>
   <sheets>
     <sheet name="Case 1" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,8 @@
     <sheet name="Case 3" sheetId="3" r:id="rId3"/>
     <sheet name="Case 4" sheetId="5" r:id="rId4"/>
     <sheet name="Case 5" sheetId="6" r:id="rId5"/>
+    <sheet name="Case 6" sheetId="7" r:id="rId6"/>
+    <sheet name="Case 7" sheetId="9" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="189">
   <si>
     <t>All the three options will have same effect</t>
   </si>
@@ -579,6 +581,296 @@
     <t>Sheetal's suggestion would decrease Gross Profit margin as profit per product reduces is lesser in than that of Asha. This is because Sheetal is suggesting to increase cost of goods sold by adding a free brush. Thus this will lead to a lower gross profit margin for Sheetal's suggestion.
 Although, the operating profit in both would be same the total expenses in both cases add up to same. Just that as per Asha's suggestion, the expense will be allocated to marketing expense whereas in Sheetal's suggestion it will be allocated to Cost of Goods sold.</t>
   </si>
+  <si>
+    <t>Company A had Rs.320 lakhs worth of finished goods and WIP in its inventory at the end of financial year 2XX8. Which of the following is closest to its inventory of finished goods and WIP at end of 2XX9?</t>
+  </si>
+  <si>
+    <t>Rs.220 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.285 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.355 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.440 lakhs</t>
+  </si>
+  <si>
+    <t>Value of Finished Goods and WIP in inventory at the end of Year 2xx8 = 320 Lakhs (Given)
+As per the generally accepted accounting principles expenditure incurred towards production of goods is retained in inventory until the goods are disposed. Thus, the line item “Changes in Inventory of WIP and finished Goods” represents the difference between opening balance and closing balance of work-in-progress and finished goods.
+Thus,
+Closing Value of Finished Goods and WIP = Opening Balance of Finished Good and WIP + Changes in Inventory of WIP and finished Goods.
+Closing Value of Finished Goods = 320 + (-35) = 285
+Thus, Closing Value of Finished Goods and WIP = 285 Lakhs</t>
+  </si>
+  <si>
+    <t>You have information that companies in the industry increased selling price of their output. However, different companies increased their prices at different rates. Which of two company is likely to have increased their price at a higher rate and why?</t>
+  </si>
+  <si>
+    <t>Company B is likely to have increased the price more as its sales grew faster than that of A</t>
+  </si>
+  <si>
+    <t>Company A is likely to have increased the price more as its cost of materials to sales ratio decreased year over year, while it remained constant for company B</t>
+  </si>
+  <si>
+    <t>Company B is likely to have increased the price more as its net profit margin increased by 23% compared to only 15% growth for Company A</t>
+  </si>
+  <si>
+    <t>Company A is likely to have increased the price more as it earned higher net profit</t>
+  </si>
+  <si>
+    <t>In order to choose the correct option, we will have to evaluate all the 4 options first.
+Option 1 is wrong because price increase cannot be judged by only looking at growth in sales. We need to also look at cost of raw material in conjunction. The ratio of cost of raw material to Operating Revenue is constant for company B in both years. This does not really imply that prices of goods were increase.
+Option 2 seems correct as the reasoning given is correct and satisfactory. Company A’s Cost of materials to Sales Ratio for 2XX8= 3024/8642 = 35%
+Company A’s Cost of materials to Sales Ratio for 2XX9= 3003/9100 = 33%
+Company B’s Cost of materials to Sales Ratio for 2xx8= 2185/6427 = 34%
+Company B’s Cost of materials to Sales Ratio for 2xx9= 2558/7524 = 34%
+When sales and cost of materials both rise, like for company B, it can be implied that the sales increased due to the increase in sale of number of units. But like for company A, where sales go up but cost of materials remains flat or goes down, it can be implied that sales increased due to increase in price per unit.
+Option 3 and 4 are incorrect because net profit is not the right metric to evaluate the growth in sales. Net profit is also affected by other factors like depreciation, taxes etc.</t>
+  </si>
+  <si>
+    <t>Which of the following is closest to the difference between EBITDA margin ratios for Company A and Company B for the 2XX9? (1 basis point or bps equals 0.01%)</t>
+  </si>
+  <si>
+    <t>Which of the two companies have higher level of financial leverage?</t>
+  </si>
+  <si>
+    <t>Both the companies have very similar margins</t>
+  </si>
+  <si>
+    <t>Company A’s EBITDA margin is 427 bps higher than Company B’s EBITDA margin</t>
+  </si>
+  <si>
+    <t>Company B’s EBITDA margin is 450 bps higher than Company A’s EBITDA margin</t>
+  </si>
+  <si>
+    <t>Company A’s EBITDA margin is 518 bps higher than Company B’s EBITDA margin</t>
+  </si>
+  <si>
+    <t>EBITDA stands for Earnings Before Interest, Taxes, Depreciation, and Amortization and is a metric used to evaluate a company’s operating performance. Interest Expense is also expressed as finance cost in some cases.
+EBITDA = Net Income + Interest Expense + Taxes + Depreciation and Amortization
+EBITDA Margin = EBITDA/Sales
+EBITDA for Company A = 2763.1 + 180.4 + 1330 + 241.2 = 4514.7
+EBITDA Margin for Company A = 4514.7/9100 = 49.61%
+EBITDA for Company B = 1962.8 + 195.2 + 966.8 + 218.6 = 3343.4
+EBITDA Margin for Company B = 3343.4/7524 = 44.43%
+Difference in EBITDA Margin = 49.61% - 44.43% = 5.18%
+Thus, the difference in EBITDA margin is 518 basis points.</t>
+  </si>
+  <si>
+    <t>Company A has higher financial leverage as it has higher level of debt</t>
+  </si>
+  <si>
+    <t>Company A has higher financial leverage as it has higher Debt / Asset ratio</t>
+  </si>
+  <si>
+    <t>Company B has higher financial leverage as it has higher Debt / Asset ratio</t>
+  </si>
+  <si>
+    <t>Company B has higher financial leverage as it has higher finance cost</t>
+  </si>
+  <si>
+    <t>The best way to compute financial leverage of a company is to calculate its Debt/Asset Ratio
+Debt/Asset Ratio for company A = 1640.5/4687 = 35%
+Debt/Asset Ratio for company B = 1626.8/4067 = 40%
+Thus, the debt level of company B is more and thus it has more financial leverage</t>
+  </si>
+  <si>
+    <t>Q5</t>
+  </si>
+  <si>
+    <t>Q6</t>
+  </si>
+  <si>
+    <t>Which of the following is closest to operating profit of Company B for the year ending 2XX9?</t>
+  </si>
+  <si>
+    <t>Rs.2,929.6 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.3,124.8 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.3,343.4 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.3,945.5 lakhs</t>
+  </si>
+  <si>
+    <t>Operating Profit, also called as EBIT is the Net Profit + Interest + Taxes
+Operating Profit for Company B = 1962.8 + 966.8 + 195.2 = 3124.8</t>
+  </si>
+  <si>
+    <t>Company A has a higher return on equity (ROE) compared to Company B. Which of the following combination of factors have favourably contributed to the higher ROE?</t>
+  </si>
+  <si>
+    <t>Higher net profit margin and higher activity ratio</t>
+  </si>
+  <si>
+    <t>Higher net profit margin, higher activity ratio and lower financial leverage</t>
+  </si>
+  <si>
+    <t>Higher net profit margin, higher activity ratio and higher financial leverage</t>
+  </si>
+  <si>
+    <t>Higher net profit margin</t>
+  </si>
+  <si>
+    <t>According to the DuPont analysis, ROE is broken up into three parts: Profit margin, Asset Turnover (i.e. Activity Ratio) and Equity Multiplier (Financial Leverage)
+Let’s calculate the ROE for both companies
+Profit Margin (A) = PAT/Net Sales
+Asset Turnover (B) = Sales/Fixed Assets
+Equity Multiplier (C) = Fixed Assets/ Net Worth
+ROE = A * B * C
+Company A
+(A): 2763.1/9100 = 0.3036
+(B): 9100/2412 = 3.7728
+(C): 2412/3046.6 = 0.7917
+ROE: 0.3036 * 3.7728 *0.7917 = 0.9068 =90.68%
+Company B
+(A): 1962.8/7254 = 0.2705
+(B): 7524/2186 = 3.4419
+(C): 2186/2440.2 = 0.8958
+ROE: 0.2705 * 3.4419 * 0.8958 = 0.8340 = 83.40%
+From the above calculation, we can see that ROE for company A is better and the metrics Net Profit Margin and Asset Turnover are better than that of Company B.</t>
+  </si>
+  <si>
+    <t>Which of the following is closest to the capital expenditure incurred by the company in 2XX7?</t>
+  </si>
+  <si>
+    <t>Which of the following is closest to the estimated revenue for 2XX8, if revenue is expected to grow at the same rate at which it grew in 2XX7?</t>
+  </si>
+  <si>
+    <t>The company expects that the revenue of 2XX8 is likely to be Rs.9,500 lakhs. It further estimates 25 bps decrease in EBITDA margin compared to previous year. Which of the following is closest to the estimated EBITDA for 2XX8 as per the company guidance?</t>
+  </si>
+  <si>
+    <t>The company also estimates that its networking capital ratio (i.e. net working capital as a % of revenue) in 2XX8 is likely to remain same compared to previous year. Which of the following is closest to increase / (decrease) in working capital, if the expected revenue of 2XX8 is Rs.9,500 lakhs?</t>
+  </si>
+  <si>
+    <t>The company is expected to repay Rs.200 lakhs of debt on the first day of financial year 2XX8. Assuming the company’s average interest rate remains unchanged, which of the following is the closest to the expected finance cost for 2XX8?</t>
+  </si>
+  <si>
+    <t>The profit for 2XX8 is estimated to be Rs.3,200 lakhs and the company is expected to pay an interim dividend of Rs.900 lakhs and a special dividend of Rs.1,000 lakhs during the year. No other dividend, shares buy back or issue of shares are expected. Which of the following is the closest to the estimated book value of equity at the end of 2XX8?</t>
+  </si>
+  <si>
+    <t>Rs.5.0 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.6.2 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.241.2 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.246.2 lakhs</t>
+  </si>
+  <si>
+    <t>Rs. 9,100 lakhs</t>
+  </si>
+  <si>
+    <t>Rs. 9,558 lakhs</t>
+  </si>
+  <si>
+    <t>Rs. 9,582 lakhs</t>
+  </si>
+  <si>
+    <t>Rs. 9,614 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.2,647 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.2,860 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.4,475 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.4,689 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.0.0 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.100.0 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.275.0 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.400.0 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.144 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.172 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.180 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.200 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.1,300 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.4,347 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.5,347 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.6,247 lakhs</t>
+  </si>
+  <si>
+    <t>Capital Expenditure for the company = Ending Fixed Assets – Beginning Fixed Assets + Depreciation and Amortization
+Capital Expenditure for the company in Year 2xx7 = 2412 – 2407 + 241.2 = 246.2</t>
+  </si>
+  <si>
+    <t>Growth Rate for Revenue from 2xx6 to 2xx7 = (Sales of 2xx7/Sales of 2xx6)-1 = (9100/8642)-1 = 0.0529 = 5.29%
+Now if Sales grow at same rate, expected sales is Year 2xx8 = (Sales in 2xx7) * (1 + growth rate)
+Expected sales in 2xx8 = 9100 * (1+5.29%) = 9100 * (1.0529) = 9581.39
+Thus, expected sales are Rs. 9582 Lakhs</t>
+  </si>
+  <si>
+    <t>First, lets calculate the EBITDA margin for Year 2xx7
+EBITDA = Net Income + Interest Expense + Taxes + Depreciation and Amortization
+EBITDA for Company = 2763.1 + 180.4 + 1330 + 241.2 = 4514.7
+EBITDA Margin = EBITDA/Sales
+EBITDA Margin for Company = 4514.7/9100 = 49.61%
+Now company expects the margin to decrease by 25 bps meaning the margin will be 49.36% (49.61% - 0.25%)
+Expected Sales are 9500 Lakhs
+Therefore, Expected EBITDA = 9500 * 0.4936 = 4689.2 Lakhs</t>
+  </si>
+  <si>
+    <t>First, let’s calculate the net working Capital as a % of Revenue for Year 2xx7
+Ratio = 2275/9100 = 0.25 = 25%
+If the Ratio remains the same and the expected Sales for 2xx8 are 9500, the networking capital for year 2xx8 will be:
+9500 * 0.25 = 2375
+There change is working capital is 100 (2375 – 2275)</t>
+  </si>
+  <si>
+    <t>First, lets calculate the average interest rate for year 2xx7.
+Interest Rate = Finance Cost/Total Capital = 180.4/4687 = 3.84%
+Now, if the company pays off 200 Lakhs worth of debt on the first day of Year 2xx8 and the average interest rate remains the same, the scenario would look as follows:
+Total Capital = Total Capital as on Year 2xx7 – 200 = 4687 – 200 = 4487
+Interest Rate of 3.84% on 4487 = 4487 * 0.0384 = 172.03
+Thus, Option B is correct</t>
+  </si>
+  <si>
+    <t>Ending Book Value of Equity = Beginning Book Value of Equity + Net Income – Dividends Paid
+Ending Book Value of Equity for Company = 3046.6 + 3200 – 1900 = 4346.6 Lakhs
+Thus estimated book value of equity at the end of year 2xx8 = 4347 Lakhs</t>
+  </si>
+  <si>
+    <t>IMG: Case 7.png</t>
+  </si>
+  <si>
+    <t>IMG: Case 6.png</t>
+  </si>
 </sst>
 </file>
 
@@ -587,10 +879,16 @@
   <numFmts count="1">
     <numFmt numFmtId="8" formatCode="&quot;₹&quot;\ #,##0.00;[Red]&quot;₹&quot;\ \-#,##0.00"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1024,27 +1322,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D596250-E0EC-41F6-BE6F-BD0A07A909DD}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="155.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="132.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="155.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="132.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B2" s="2"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>64</v>
       </c>
@@ -1070,7 +1368,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="261" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="270" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>75</v>
       </c>
@@ -1096,7 +1394,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="319" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="330" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>77</v>
       </c>
@@ -1122,7 +1420,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="348" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="375" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>79</v>
       </c>
@@ -1148,7 +1446,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="333.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="345" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>81</v>
       </c>
@@ -1182,24 +1480,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80FEDD49-34CC-4B42-AED5-3DAD0ACA7221}">
   <dimension ref="A1:M33"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="126" customWidth="1"/>
-    <col min="3" max="3" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="105.7265625" customWidth="1"/>
+    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="105.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>64</v>
       </c>
@@ -1225,7 +1523,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="217.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="225" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>75</v>
       </c>
@@ -1251,7 +1549,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="232" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="240" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>77</v>
       </c>
@@ -1277,7 +1575,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="145" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="150" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>79</v>
       </c>
@@ -1303,7 +1601,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="87" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>81</v>
       </c>
@@ -1329,7 +1627,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="33" spans="13:13" x14ac:dyDescent="0.35">
+    <row r="33" spans="13:13" x14ac:dyDescent="0.25">
       <c r="M33" s="1">
         <f>FV(12%,1,0,-330)</f>
         <v>369.6</v>
@@ -1343,23 +1641,23 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{016B9E16-9F58-446C-8FE7-F7028D7547DC}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="90.54296875" customWidth="1"/>
-    <col min="8" max="8" width="117.26953125" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="90.5703125" customWidth="1"/>
+    <col min="8" max="8" width="117.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>64</v>
       </c>
@@ -1385,7 +1683,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="232" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="270" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>75</v>
       </c>
@@ -1411,7 +1709,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="165" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>77</v>
       </c>
@@ -1437,7 +1735,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="290" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="330" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>79</v>
       </c>
@@ -1463,7 +1761,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="261" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="270" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>81</v>
       </c>
@@ -1489,25 +1787,25 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="5"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
     </row>
   </sheetData>
@@ -1518,20 +1816,20 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EBCDB2F-626E-4298-9A86-1618491D5242}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="145.1796875" customWidth="1"/>
-    <col min="6" max="6" width="12.54296875" customWidth="1"/>
-    <col min="8" max="8" width="75.54296875" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="145.140625" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" customWidth="1"/>
+    <col min="8" max="8" width="75.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>64</v>
       </c>
@@ -1557,7 +1855,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="116" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>75</v>
       </c>
@@ -1583,7 +1881,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="116" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>77</v>
       </c>
@@ -1609,7 +1907,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>79</v>
       </c>
@@ -1635,7 +1933,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="300" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>81</v>
       </c>
@@ -1669,20 +1967,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A23A3889-F024-4DED-9AE6-26A473053FC8}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="138.26953125" customWidth="1"/>
-    <col min="3" max="6" width="19.90625" style="13" customWidth="1"/>
-    <col min="8" max="8" width="63.7265625" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="138.28515625" customWidth="1"/>
+    <col min="3" max="6" width="19.85546875" style="13" customWidth="1"/>
+    <col min="8" max="8" width="63.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>64</v>
       </c>
@@ -1708,7 +2006,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="165" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>75</v>
       </c>
@@ -1734,7 +2032,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="145" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" ht="165" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>77</v>
       </c>
@@ -1760,7 +2058,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="246.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="270" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>79</v>
       </c>
@@ -1784,7 +2082,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" ht="165" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>81</v>
       </c>
@@ -1806,6 +2104,415 @@
       </c>
       <c r="H7" s="12" t="s">
         <v>112</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB9CB08A-8EFD-4E9F-AAF5-BB242D089D92}">
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="82.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="76.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="225" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="315" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="210" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="105" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="360" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>150</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0248B61-3F3C-4B55-A7B1-1529F237D16C}">
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="84" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="76.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="120" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="150" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="105" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="135" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>186</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Case 8, 9, 10, 11
</commit_message>
<xml_diff>
--- a/Data/Sample.xlsx
+++ b/Data/Sample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PyCode\nism\quiz_app\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07703D48-C3EB-4210-81CA-C416C1CC412C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73DD2EDD-7DAA-4296-AC92-4E8CB1EE4FD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="5" xr2:uid="{B3B2EAEB-3D4F-44E9-A7BC-7C78BD8AFC15}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="2" activeTab="10" xr2:uid="{B3B2EAEB-3D4F-44E9-A7BC-7C78BD8AFC15}"/>
   </bookViews>
   <sheets>
     <sheet name="Case 1" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,10 @@
     <sheet name="Case 5" sheetId="6" r:id="rId5"/>
     <sheet name="Case 6" sheetId="7" r:id="rId6"/>
     <sheet name="Case 7" sheetId="9" r:id="rId7"/>
+    <sheet name="Case 8" sheetId="10" r:id="rId8"/>
+    <sheet name="Case 9" sheetId="11" r:id="rId9"/>
+    <sheet name="Case 10" sheetId="12" r:id="rId10"/>
+    <sheet name="Case 11" sheetId="13" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="291">
   <si>
     <t>All the three options will have same effect</t>
   </si>
@@ -870,6 +874,385 @@
   </si>
   <si>
     <t>IMG: Case 6.png</t>
+  </si>
+  <si>
+    <t>IMG: Case 8.png</t>
+  </si>
+  <si>
+    <t>PE ratio for Company B is higher than that of Company A. Which of the following are plausible reasons to justify such higher PE ratio of Company B?</t>
+  </si>
+  <si>
+    <t>Which of these two companies appear cheaper based on PEG ratio? Use the expected growth rate for 2XX9 for the calculation.</t>
+  </si>
+  <si>
+    <t>Which of the following is closest to the market value of equity (i.e., market capitalization) of Company A?</t>
+  </si>
+  <si>
+    <t>The market cap of Company B based on its last traded price is Rs.36,000 lakhs. Which of the following is closest to its EV/EBITDA based on forecast for 2XX9?</t>
+  </si>
+  <si>
+    <t>The average PE ratio of peers in the industry is 16x based on 2XX9 earnings. The analyst believes that Company B deserves to trade at 20% premium compared to its peers because of its low risk and high growth potential. Which of the following is closest to the fair price of its share?</t>
+  </si>
+  <si>
+    <t>The analysts’ estimate of the fair EV/EBITDA multiple for Company A is 8.5x. Which of the following is closest to the fair value of the company’s equity?</t>
+  </si>
+  <si>
+    <t>EPS growth rate for Company B is higher than EPS growth rate for Company A and higher growth justifies higher PE ratio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Company B is relative smaller company, and the smaller base justifies higher PE ratio </t>
+  </si>
+  <si>
+    <t>Company B has high financial leverage which justifies higher PE ratio</t>
+  </si>
+  <si>
+    <t>None of the above statements are true</t>
+  </si>
+  <si>
+    <t>Company A is cheaper as its PEG ratio is 1.05x compared to 0.91x for Company B</t>
+  </si>
+  <si>
+    <t>Company B is cheaper as its PEG ratio is 0.91x compared to 1.05x for Company A</t>
+  </si>
+  <si>
+    <t>Company A is cheaper as its PEG ratio is 2.91x compared to 1.07x for Company B</t>
+  </si>
+  <si>
+    <t>Company B is cheaper as its PEG ratio is 1.07x compared to 2.91x for company A</t>
+  </si>
+  <si>
+    <t>Rs.3,046 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.30,000 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.42,600 lakhs</t>
+  </si>
+  <si>
+    <t>None of the above</t>
+  </si>
+  <si>
+    <t>8.17x</t>
+  </si>
+  <si>
+    <t>8.74x</t>
+  </si>
+  <si>
+    <t>9.14x</t>
+  </si>
+  <si>
+    <t>9.54x</t>
+  </si>
+  <si>
+    <t>Rs.428.7</t>
+  </si>
+  <si>
+    <t>Rs.514.8</t>
+  </si>
+  <si>
+    <t>Rs.617.8</t>
+  </si>
+  <si>
+    <t>Rs.643.6</t>
+  </si>
+  <si>
+    <t>Rs.38,943 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.40,415 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.41,886 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.42,224 lakhs</t>
+  </si>
+  <si>
+    <t>Lets evaluate all 4 statements.
+Option 1 seems correct. EPS growth rates for companies A and B are 14.7% {(19.5/17)-1} and 20.14% {(32.2/26.8)-1} respectively if calculated from the rates given. Higher EPS growth rate commands for a higher PE
+Option 2 is incorrect because only size does not matter in determining the fair PE of a company. Growth rate is what needs to be taken into account
+Option 3 is wrong because higher financial leverage ratio should imply for a lower PE and not a higher PE.</t>
+  </si>
+  <si>
+    <t>PEG Ratio = PE Ratio/Growth Rate
+Growth Rate for company = Growth rate in EPS = (EPS for this year/EPS of Previous Year) - 1
+Growth Rate for Company A = (19.5/17)- 1 = 14.7%
+Growth Rate for Company B = (32.2/26.8)- 1 = 20.14%
+PEG Ratio of Company A = 15.4/14.7 = 1.047 = 1.05
+PEG Ratio of Company B = 18.2/20.14 = 0.9036 = 0.91
+PEG Ratio of company B is lower. Lower the PEG ratio, the better as it implies a lower price of stock.
+Thus, Option B is correct.</t>
+  </si>
+  <si>
+    <t>EV or Enterprise Value of a Company = Market Value of Equity + Market Value of Debt – Cash and Equivalents
+EV of Company B = 36000 + 1626.8 – 57 = 37569.8
+EBITA of Company B = 3938.8
+EV/EBITDA of the company = 37569.8/3938.8 = 9.5383 = 9.54
+Thus, Option D is correct</t>
+  </si>
+  <si>
+    <t>Market Cap of Company = PE Ratio * Earnings per Share * No of Outstanding Shares
+No of Outstanding Shares = Total Profit/ EPS = 2763.1/19.5 = 141.69
+Market Cap of Company = 15.4 * 19.5 * 141.69 = 42549 Lakhs
+Thus, Option C is Correct</t>
+  </si>
+  <si>
+    <t>Expected EPS of Company B in 2xx9 = 32.2
+PE Ratio of Peers = 16x
+Market Price without premium = 16 * 32.2 = 515.2
+Now, analysts believe that the company deserves to trade a 20% premium;
+Thus, Market Price with Premium = 515.2 * (1+20%) = 515.2 * 1.2 = 618.24
+Thus, Option C being the closest is the correct answer</t>
+  </si>
+  <si>
+    <t>EV or Enterprise Value of a Company = Market Value of Equity + Market Value of Debt – Cash and Equivalents
+According to the fair EV/EBITDA multiple of 8.5, the EV of company A should be
+= 8.5 * 4754.6 = 40414.1
+Substituting all other values in the EV formula, we can find the fair value of Equity
+40414.1 = Fair Market Value of Equity + 1640.5 – 169
+Thus, Fair Market Value of Equity = 40414.1 – 1640.5 + 169 = 38942.6
+Thus, Fair Market value of Equity is 38943 Lakhs and hence Option A is correct.</t>
+  </si>
+  <si>
+    <t>The AGM of the company approved dividend for the recently concluded year and it was just paid. If the dividend is expected to grow at a constant rate of 5%, which of the following is closest to the fair price of the share, assuming cost of equity of 12%?</t>
+  </si>
+  <si>
+    <t>Which of the following is closest to the free cash flow to firm for 2XX8?</t>
+  </si>
+  <si>
+    <t>Based on the following information, calculate the cost of equity of the company? Risk free rate: 6% Expected return from the market: 10% Beta of the company: 1.2</t>
+  </si>
+  <si>
+    <t>The fair value of total assets of the company is expected to be Rs.12,000 lakhs while the liabilities are worth the same as shown in the balance sheet. If the cost of equity is 12% and cost of debt (net of tax) is 8%, which of the following is closest to the weighted average cost of capital?</t>
+  </si>
+  <si>
+    <t>The FCFF of the company for next year is estimated at 2,000 lakhs. It is expected to grow at 10% in the year after that and is expected to grow at 5% perpetually post that. If the weighted average capital is 11.0%, which of the following is closest to the fair value of the firm (Enterprise value)?</t>
+  </si>
+  <si>
+    <t>Rs.113</t>
+  </si>
+  <si>
+    <t>Rs.142</t>
+  </si>
+  <si>
+    <t>Rs.194</t>
+  </si>
+  <si>
+    <t>Rs.204</t>
+  </si>
+  <si>
+    <t>Rs.1,624 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.1,677 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.1,747 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.1,800 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.33,333 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.34,835 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.42,087 lakhs</t>
+  </si>
+  <si>
+    <t>Rs.42,700 lakhs</t>
+  </si>
+  <si>
+    <t>IMG: Case 9.png</t>
+  </si>
+  <si>
+    <t>According to Gordon growth Model;
+Value of Share = D1/(k-g)
+Where;
+D1 = Dividend per share in Year 1
+K = Cost of Equity
+G = Growth Rate
+Dividend in Year 0 = EPS * Payout Ratio = 17 * 0.8 = 13.6
+D1 = D0 * (1+g)
+D1 = 13.6 * 1.05
+D1 = 14.28
+Value of Share = 14.28/(0.12-0.05) = 14.28/0.07 = 204
+Thus, Option D is correct</t>
+  </si>
+  <si>
+    <t>Free Cash Flow to Firm = Operating Cash Flow – Capital Expenditure – Tax benefit on interest payments
+Tax benefit on interest payments is the tax saved due to the interest cost. It is calculated as Interest Cost * Tax rate viz. 175.8 * 0.3 for this case i.e 52.74
+Free Cash Flow to Firm = 4200 – 2400 – 52.74 = 1747.26
+Thus, Free Cash Flow to Firm is 1747 Lakhs and thus Option C is correct</t>
+  </si>
+  <si>
+    <t>According the capital asset pricing model, 
+Ke = Rf + β * (Rm – Rf)
+Thus,
+Ke = 6% + 1.2*(10%-6%)
+Ke = 6% + 1.2*(4%)
+Ke = 6% + 4.8%
+Ke = 10.8%
+Thus, Option B is correct</t>
+  </si>
+  <si>
+    <t>Fair Value of Debt = 1598
+Fair Value of Equity = 12,000
+Total Fair Value = 1598 + 12000 = 13598
+Proportion of Debt = 1598/13598 = 11.75%
+Proportion of Equity = 88.25%
+Weighted Average Cost of Capital = (Proportion of Debt * Cost of Debt) + (Proportion of Equity * Cost of Equity)
+= (11.75% * 8%) + (12% * 88.25%)
+= 0.0094 + 0.1059
+= 0.1153 or 11.53%
+Thus, Option D is correct</t>
+  </si>
+  <si>
+    <t>Fair Value of the Firm = Sum of present values of FCFF in the future years
+FCFF in Year 1 = 2000
+FCFF in Year 2 = 2000 * 1.1 (As per 10% growth rate given)
+Now, PV of all future FCFF from Year 2 onwards can be calculated because growth rate becomes constant.
+PV of all future FCFF from Year 2 in Year 1 = FCFF of Year 2/(Discount Rate – Growth Rate) = 2200/(0.11-0.05) = 2200/0.06 = 36,666
+Now we have FCFF Values in Year 1, which we need to discount back to today viz, Year 0.
+PV of All FCFF = PV of FCFF in Year 1 + PV of all future FCFF from Year 2 in Year 0
+PV of All FCFF = 2000/1.11 + 36666/1.11 = 1801 + 33033 = 34834
+Thus, Option B is correct</t>
+  </si>
+  <si>
+    <t>IMG: Case 10.png</t>
+  </si>
+  <si>
+    <t>Based on the given weekly candlestick chart of Oceanic Shipping Co. Ltd, a bullish engulfing pattern is observed during which of the following periods?</t>
+  </si>
+  <si>
+    <t>Based on visual comparison with the Nifty index (Dark Red line), Oceanic Shipping appears to outperform the benchmark during which period?”</t>
+  </si>
+  <si>
+    <t>Around which period did the On-Balance Volume (OBV) indicator give a clear buy signal?</t>
+  </si>
+  <si>
+    <t>Which of the following moving average patterns has generally remained valid from January 2022 to December 2025? (EMA - Exponential Moving Average)</t>
+  </si>
+  <si>
+    <t>The bullish engulfing pattern is identified when a large green candle completely engulfs the real body of the preceding red candle after a decline.
+In the chart, this formation appears during the week ending 10 June 2022, following a sharp fall in April–May 2022. The candle forms near a swing low, increasing its reversal significance. Trading volume during this week is also relatively higher, supporting buying interest. The subsequent weeks show follow-through upward movement, confirming the validity of the bullish engulfing signal.</t>
+  </si>
+  <si>
+    <t>From around June 2023, Oceanic Shipping begins to rise at a steeper pace than the Nifty index, indicating stronger price momentum. While the Nifty moves up gradually, Oceanic Shipping records faster higher highs and shallower corrections, suggesting relative strength.
+This phase continues through most of 2024, during which Oceanic Shipping consistently stays above its rising moving averages and advances more sharply than the index. The widening gap between the stock’s price movement and the index reflects apparent outperformance. Hence, based on visual comparison, Oceanic Shipping appears to outperform the Nifty from mid-2023 to late-2024.</t>
+  </si>
+  <si>
+    <t>Around June 2022, the price action shows a clear base formation after a sharp decline. During this phase, trading volumes expand noticeably, indicating accumulation by informed participants.
+The On-Balance Volume (OBV), being a volume-based indicator, would have started rising even before the price breakout, signaling strengthening buying pressure. Soon after, the price breaks above the consolidation range and begins a sustained uptrend. This alignment of rising OBV and improving price structure confirms a buy signal around June 2022.</t>
+  </si>
+  <si>
+    <t>NOTE : When the stock is in an uptrend, Price &gt; 13 EMA &gt; 21EMA &gt; 34 EMA. In a bull market, the price usually takes support around its 34 EMA. When all 3 averages are rising and move away from each other, it indicates a strong bull market.
+When the stock is in a downtrend, Price &lt; 13 EMA &lt; 21EMA &lt; 34 EMA. The price generally will tend to resist around its 34 EMA.
+Moving averages plotted in different colors (green, orange, yellow lines). These represent short-, medium-, and longer-term EMAs
+In the above question : From January 2022 to December 2025, the chart exhibits a sustained upward trend with higher highs and higher lows. During most of this period, the short-term 13 EMA remains above the 21 EMA, and the 21 EMA stays above the long-term 34 EMA, indicating bullish momentum. Although there are brief corrections where the EMAs converge, the bullish alignment is quickly re-established.
+This persistent stacking of shorter EMAs above longer EMAs reflects continued buying interest and trend strength. Hence, the moving average pattern that has generally held good is 13 EMA &gt; 21 EMA &gt; 34 EMA.</t>
+  </si>
+  <si>
+    <t>Week ending 10 June 2022</t>
+  </si>
+  <si>
+    <t>Week ending 30 September 2022</t>
+  </si>
+  <si>
+    <t>Week ending 23 June 2023</t>
+  </si>
+  <si>
+    <t>January 2022 to March 2022</t>
+  </si>
+  <si>
+    <t>August 2022 to February 2023</t>
+  </si>
+  <si>
+    <t>June 23 to Dec 24</t>
+  </si>
+  <si>
+    <t>34 EMA &lt; 21 EMA &lt; 13 EMA</t>
+  </si>
+  <si>
+    <t>21 EMA &gt; 34 EMA &gt; 13 EMA</t>
+  </si>
+  <si>
+    <t>13 EMA &gt; 21 EMA &gt; 34 EMA</t>
+  </si>
+  <si>
+    <t>Week ending 12 January 2024</t>
+  </si>
+  <si>
+    <t>January 2025 to December 2025</t>
+  </si>
+  <si>
+    <t>34 EMA &gt; 21 EMA &gt; 13 EMA</t>
+  </si>
+  <si>
+    <t>IMG: Case 11.png</t>
+  </si>
+  <si>
+    <t>Which of the following regarding RSI is most likely to be true?</t>
+  </si>
+  <si>
+    <t>Which of the following regarding RSI is NOT likely to be true?</t>
+  </si>
+  <si>
+    <t>Which of the following regarding MACD is most likely to be true?</t>
+  </si>
+  <si>
+    <t>Which of the following regarding MACD is not likely to be true?</t>
+  </si>
+  <si>
+    <t>The RSI shows a bullish divergence around the last week of February 2025.</t>
+  </si>
+  <si>
+    <t>In a strong trend, from Dec 23 - Sep 24, RSI continues to remain overbought.</t>
+  </si>
+  <si>
+    <t>The RSI shows a bearish divergence around the second week of September 2023.</t>
+  </si>
+  <si>
+    <t>The RSI can take a value above 100 in a very strong bull market.</t>
+  </si>
+  <si>
+    <t>The RSI value can fall below 40 in a strong bull market.</t>
+  </si>
+  <si>
+    <t>Nifty makes a new high around Sep 2024, but the RSI fails to make a new high.</t>
+  </si>
+  <si>
+    <t>It is normal to observe an RSI value below 30 in an extremely bearish market</t>
+  </si>
+  <si>
+    <t>The RSI measures the speed and magnitude of a security's recent price</t>
+  </si>
+  <si>
+    <t>Nifty makes a high in Sep’24 but MACD doesn’t, indicating a negative divergence.</t>
+  </si>
+  <si>
+    <t>One can initiate a long trade if the MACD moves over the zero line.</t>
+  </si>
+  <si>
+    <t>The MACD trades between 0 and 100 most of the time.</t>
+  </si>
+  <si>
+    <t>The MACD is generally considered as a lead indicator.</t>
+  </si>
+  <si>
+    <t>The MACD slow line is generated from the 9 EMA of the fast line.</t>
+  </si>
+  <si>
+    <t>With both the lines rising, buy when the fast MACD crosses over the slow MACD.</t>
+  </si>
+  <si>
+    <t>When the MACD makes a double top or a double bottom, a trend reversal is likely.</t>
+  </si>
+  <si>
+    <t>The MACD gave a buy signal in the first week of Oct 2024</t>
   </si>
 </sst>
 </file>
@@ -941,7 +1324,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -985,6 +1368,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1477,6 +1863,302 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2A07478-22A2-4F3D-BB40-6F5280FB117B}">
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="84" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="76.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="120" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>267</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="150" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>263</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="135" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="C6" s="19">
+        <v>44713</v>
+      </c>
+      <c r="D6" s="19">
+        <v>45139</v>
+      </c>
+      <c r="E6" s="19">
+        <v>45292</v>
+      </c>
+      <c r="F6" s="19">
+        <v>45778</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="285" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>264</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>265</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>266</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>257</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{489BEFBF-44C3-4BCB-9DBE-5C0EC38F204C}">
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="84" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="76.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="135" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="H4" s="12"/>
+    </row>
+    <row r="5" spans="1:8" ht="120" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>280</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>282</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H5" s="12"/>
+    </row>
+    <row r="6" spans="1:8" ht="120" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>283</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>284</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>285</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>286</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H6" s="12"/>
+    </row>
+    <row r="7" spans="1:8" ht="135" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>274</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>287</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>289</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>290</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="H7" s="12"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80FEDD49-34CC-4B42-AED5-3DAD0ACA7221}">
   <dimension ref="A1:M33"/>
@@ -2518,4 +3200,386 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{142F5273-98E1-48DE-9B14-EC6B8B03BF66}">
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="84" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="76.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="195" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="195" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>204</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="120" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="120" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="165" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>225</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20E8462A-7253-4269-9E64-ABAA098AE66C}">
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="84" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="76.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="225" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="135" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>235</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>236</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>237</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="150" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="C6" s="15">
+        <v>7.1999999999999995E-2</v>
+      </c>
+      <c r="D6" s="15">
+        <v>0.108</v>
+      </c>
+      <c r="E6" s="15">
+        <v>0.12</v>
+      </c>
+      <c r="F6" s="15">
+        <v>0.18</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="210" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>229</v>
+      </c>
+      <c r="C7" s="15">
+        <v>0.08</v>
+      </c>
+      <c r="D7" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="E7" s="15">
+        <v>0.11</v>
+      </c>
+      <c r="F7" s="15">
+        <v>0.115</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="240" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>239</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>240</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>248</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>